<commit_message>
Weekly update Thu 06/04/2026
</commit_message>
<xml_diff>
--- a/VDC Short Term Kanban.xlsx
+++ b/VDC Short Term Kanban.xlsx
@@ -28860,7 +28860,7 @@
         <v>Medium</v>
       </c>
       <c r="G487" t="str">
-        <v>Amber Webb;Nicholas Ambrosino;Robert White</v>
+        <v>Amber Webb;Robert White</v>
       </c>
       <c r="H487" t="str">
         <v>Nicholas Ambrosino</v>
@@ -63410,7 +63410,7 @@
         <v>Medium</v>
       </c>
       <c r="G487" t="str">
-        <v>ea3a7b10-e540-4727-a6c2-523e99fee36e;f23519cd-6d4d-4cf3-8c1d-dcef0734dd79;4572dfb3-e99e-4bad-9d67-d344178b2d4b</v>
+        <v>ea3a7b10-e540-4727-a6c2-523e99fee36e;4572dfb3-e99e-4bad-9d67-d344178b2d4b</v>
       </c>
       <c r="H487" t="str">
         <v>f23519cd-6d4d-4cf3-8c1d-dcef0734dd79</v>

</xml_diff>

<commit_message>
Weekly update Mon 06/08/2026
</commit_message>
<xml_diff>
--- a/VDC Short Term Kanban.xlsx
+++ b/VDC Short Term Kanban.xlsx
@@ -428,7 +428,7 @@
         <v>VDC Short Term Kanban</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-06-04</v>
+        <v>2026-06-08</v>
       </c>
     </row>
   </sheetData>
@@ -440,7 +440,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S595"/>
+  <dimension ref="A1:S596"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -28778,7 +28778,7 @@
         <v>Modeling;Construction Phase;Process Mechanical Modeling</v>
       </c>
       <c r="S485" t="str">
-        <v>Adjusting walls based on conversation last week</v>
+        <v>Walls adjusted, finishing up roof modeling.</v>
       </c>
     </row>
     <row r="486">
@@ -28837,7 +28837,7 @@
         <v>Modeling;Construction Phase;Process Mechanical Modeling</v>
       </c>
       <c r="S486" t="str">
-        <v>RFIs have been submitted and returned, working through them.</v>
+        <v>RFIs have been submitted and returned, working through them. Approximately 50% complete.</v>
       </c>
     </row>
     <row r="487">
@@ -28896,7 +28896,7 @@
         <v>Modeling;Construction Phase;Process Mechanical Modeling</v>
       </c>
       <c r="S487" t="str">
-        <v>Basement modeling complete, working through first level. Approx 50% modeled on Lev 1.</v>
+        <v>Basement modeling complete, working through first level. Approx 60% modeled on Lev 1.</v>
       </c>
     </row>
     <row r="488">
@@ -32711,7 +32711,7 @@
         <v/>
       </c>
       <c r="M555" t="str">
-        <v>false</v>
+        <v>true</v>
       </c>
       <c r="N555" t="str">
         <v/>
@@ -33297,13 +33297,13 @@
         <v>Congregation B'Nai Israel Logistics</v>
       </c>
       <c r="C566" t="str">
-        <v>Done</v>
+        <v>Doing</v>
       </c>
       <c r="D566" t="str">
         <v/>
       </c>
       <c r="E566" t="str">
-        <v>Completed</v>
+        <v>Not started</v>
       </c>
       <c r="F566" t="str">
         <v>Medium</v>
@@ -33330,16 +33330,16 @@
         <v>false</v>
       </c>
       <c r="N566" t="str">
-        <v>2026-05-15</v>
+        <v/>
       </c>
       <c r="O566" t="str">
-        <v>Nicholas Ambrosino</v>
+        <v/>
       </c>
       <c r="P566" t="str">
-        <v>3/3</v>
+        <v>4/4</v>
       </c>
       <c r="Q566" t="str">
-        <v>V1 - 5.5.26;V0 - 5.1.26;V2 - 5.5.26</v>
+        <v>V1 - 5.5.26;V3 - 5.11.26;V0 - 5.1.26;V2 - 5.5.26</v>
       </c>
       <c r="R566" t="str">
         <v>Site Logistics</v>
@@ -33374,7 +33374,7 @@
         <v>2026-05-07</v>
       </c>
       <c r="J567" t="str">
-        <v>2026-06-03</v>
+        <v>2026-06-09</v>
       </c>
       <c r="K567" t="str">
         <v/>
@@ -33383,7 +33383,7 @@
         <v/>
       </c>
       <c r="M567" t="str">
-        <v>true</v>
+        <v>false</v>
       </c>
       <c r="N567" t="str">
         <v/>
@@ -33860,7 +33860,7 @@
         <v>Low Rd RFIs</v>
       </c>
       <c r="C576" t="str">
-        <v>Doing</v>
+        <v>Done</v>
       </c>
       <c r="D576" t="str">
         <v/>
@@ -34140,7 +34140,7 @@
         <v>Update Clark Logistics with new layout</v>
       </c>
       <c r="C581" t="str">
-        <v>Done</v>
+        <v>Doing</v>
       </c>
       <c r="D581" t="str">
         <v/>
@@ -34149,7 +34149,7 @@
         <v>Not started</v>
       </c>
       <c r="F581" t="str">
-        <v>Medium</v>
+        <v>Important</v>
       </c>
       <c r="G581" t="str">
         <v>Amber Webb</v>
@@ -34161,7 +34161,7 @@
         <v>2026-05-22</v>
       </c>
       <c r="J581" t="str">
-        <v/>
+        <v>2026-06-08</v>
       </c>
       <c r="K581" t="str">
         <v/>
@@ -34185,7 +34185,7 @@
         <v/>
       </c>
       <c r="R581" t="str">
-        <v>Site Logistics</v>
+        <v>Site Logistics;Preconstruction</v>
       </c>
     </row>
     <row r="582">
@@ -34362,7 +34362,7 @@
         <v>Process Mechanical Modeling</v>
       </c>
       <c r="S584" t="str">
-        <v>Waiting on Design Models</v>
+        <v>Waiting on Design Models. Michael said he talked to owner and was confident we would get something soon.</v>
       </c>
     </row>
     <row r="585">
@@ -34541,7 +34541,7 @@
         <v>FL Box Culvert show Elevations on Section Views</v>
       </c>
       <c r="C588" t="str">
-        <v>Doing</v>
+        <v>Done</v>
       </c>
       <c r="D588" t="str">
         <v/>
@@ -34587,6 +34587,9 @@
       </c>
       <c r="R588" t="str">
         <v>Coordination;Construction Phase</v>
+      </c>
+      <c r="S588" t="str">
+        <v>Sent out to project team, with all new elevations labeled</v>
       </c>
     </row>
     <row r="589">
@@ -34877,7 +34880,7 @@
         <v>Woonsocket Area C Level 1 Signoff</v>
       </c>
       <c r="C594" t="str">
-        <v>To do</v>
+        <v>Doing</v>
       </c>
       <c r="D594" t="str">
         <v/>
@@ -34898,7 +34901,7 @@
         <v>2026-06-02</v>
       </c>
       <c r="J594" t="str">
-        <v>2026-06-04</v>
+        <v>2026-06-09</v>
       </c>
       <c r="K594" t="str">
         <v/>
@@ -34945,7 +34948,7 @@
         <v>Medium</v>
       </c>
       <c r="G595" t="str">
-        <v/>
+        <v>Amber Webb</v>
       </c>
       <c r="H595" t="str">
         <v>Amber Webb</v>
@@ -34978,19 +34981,75 @@
         <v/>
       </c>
       <c r="R595" t="str">
-        <v/>
+        <v>Site Logistics;Construction Phase</v>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="str">
+        <v>uxx9CDvxYEixOsqoelK5SmUAK_4f</v>
+      </c>
+      <c r="B596" t="str">
+        <v>Glen Dr Septic As-Built</v>
+      </c>
+      <c r="C596" t="str">
+        <v>Doing</v>
+      </c>
+      <c r="D596" t="str">
+        <v/>
+      </c>
+      <c r="E596" t="str">
+        <v>Not started</v>
+      </c>
+      <c r="F596" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="G596" t="str">
+        <v>Robert White</v>
+      </c>
+      <c r="H596" t="str">
+        <v>Nicholas Ambrosino</v>
+      </c>
+      <c r="I596" t="str">
+        <v>2026-06-08</v>
+      </c>
+      <c r="J596" t="str">
+        <v/>
+      </c>
+      <c r="K596" t="str">
+        <v/>
+      </c>
+      <c r="L596" t="str">
+        <v/>
+      </c>
+      <c r="M596" t="str">
+        <v>false</v>
+      </c>
+      <c r="N596" t="str">
+        <v/>
+      </c>
+      <c r="O596" t="str">
+        <v/>
+      </c>
+      <c r="P596" t="str">
+        <v/>
+      </c>
+      <c r="Q596" t="str">
+        <v/>
+      </c>
+      <c r="R596" t="str">
+        <v>As-Built;Construction Phase</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S595"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S596"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S595"/>
+  <dimension ref="A1:S596"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -63328,7 +63387,7 @@
         <v>Modeling;Construction Phase;Process Mechanical Modeling</v>
       </c>
       <c r="S485" t="str">
-        <v>Adjusting walls based on conversation last week</v>
+        <v>Walls adjusted, finishing up roof modeling.</v>
       </c>
     </row>
     <row r="486">
@@ -63387,7 +63446,7 @@
         <v>Modeling;Construction Phase;Process Mechanical Modeling</v>
       </c>
       <c r="S486" t="str">
-        <v>RFIs have been submitted and returned, working through them.</v>
+        <v>RFIs have been submitted and returned, working through them. Approximately 50% complete.</v>
       </c>
     </row>
     <row r="487">
@@ -63446,7 +63505,7 @@
         <v>Modeling;Construction Phase;Process Mechanical Modeling</v>
       </c>
       <c r="S487" t="str">
-        <v>Basement modeling complete, working through first level. Approx 50% modeled on Lev 1.</v>
+        <v>Basement modeling complete, working through first level. Approx 60% modeled on Lev 1.</v>
       </c>
     </row>
     <row r="488">
@@ -67261,7 +67320,7 @@
         <v/>
       </c>
       <c r="M555" t="str">
-        <v>false</v>
+        <v>true</v>
       </c>
       <c r="N555" t="str">
         <v/>
@@ -67847,13 +67906,13 @@
         <v>Congregation B'Nai Israel Logistics</v>
       </c>
       <c r="C566" t="str">
-        <v>RDgWMx4cKUe-VTRRwOeAsWUADV42</v>
+        <v>J10N4yGDiUywCTAZI2lyOGUAHFjv</v>
       </c>
       <c r="D566" t="str">
         <v/>
       </c>
       <c r="E566" t="str">
-        <v>Completed</v>
+        <v>Not started</v>
       </c>
       <c r="F566" t="str">
         <v>Medium</v>
@@ -67880,16 +67939,16 @@
         <v>false</v>
       </c>
       <c r="N566" t="str">
-        <v>2026-05-15</v>
+        <v/>
       </c>
       <c r="O566" t="str">
-        <v>f23519cd-6d4d-4cf3-8c1d-dcef0734dd79</v>
+        <v/>
       </c>
       <c r="P566" t="str">
-        <v>3/3</v>
+        <v>4/4</v>
       </c>
       <c r="Q566" t="str">
-        <v>V1 - 5.5.26;V0 - 5.1.26;V2 - 5.5.26</v>
+        <v>V1 - 5.5.26;V3 - 5.11.26;V0 - 5.1.26;V2 - 5.5.26</v>
       </c>
       <c r="R566" t="str">
         <v>Site Logistics</v>
@@ -67924,7 +67983,7 @@
         <v>2026-05-07</v>
       </c>
       <c r="J567" t="str">
-        <v>2026-06-03</v>
+        <v>2026-06-09</v>
       </c>
       <c r="K567" t="str">
         <v/>
@@ -67933,7 +67992,7 @@
         <v/>
       </c>
       <c r="M567" t="str">
-        <v>true</v>
+        <v>false</v>
       </c>
       <c r="N567" t="str">
         <v/>
@@ -68410,7 +68469,7 @@
         <v>Low Rd RFIs</v>
       </c>
       <c r="C576" t="str">
-        <v>J10N4yGDiUywCTAZI2lyOGUAHFjv</v>
+        <v>RDgWMx4cKUe-VTRRwOeAsWUADV42</v>
       </c>
       <c r="D576" t="str">
         <v/>
@@ -68690,7 +68749,7 @@
         <v>Update Clark Logistics with new layout</v>
       </c>
       <c r="C581" t="str">
-        <v>RDgWMx4cKUe-VTRRwOeAsWUADV42</v>
+        <v>J10N4yGDiUywCTAZI2lyOGUAHFjv</v>
       </c>
       <c r="D581" t="str">
         <v/>
@@ -68699,7 +68758,7 @@
         <v>Not started</v>
       </c>
       <c r="F581" t="str">
-        <v>Medium</v>
+        <v>Important</v>
       </c>
       <c r="G581" t="str">
         <v>ea3a7b10-e540-4727-a6c2-523e99fee36e</v>
@@ -68711,7 +68770,7 @@
         <v>2026-05-22</v>
       </c>
       <c r="J581" t="str">
-        <v/>
+        <v>2026-06-08</v>
       </c>
       <c r="K581" t="str">
         <v/>
@@ -68735,7 +68794,7 @@
         <v/>
       </c>
       <c r="R581" t="str">
-        <v>Site Logistics</v>
+        <v>Site Logistics;Preconstruction</v>
       </c>
     </row>
     <row r="582">
@@ -68912,7 +68971,7 @@
         <v>Process Mechanical Modeling</v>
       </c>
       <c r="S584" t="str">
-        <v>Waiting on Design Models</v>
+        <v>Waiting on Design Models. Michael said he talked to owner and was confident we would get something soon.</v>
       </c>
     </row>
     <row r="585">
@@ -69091,7 +69150,7 @@
         <v>FL Box Culvert show Elevations on Section Views</v>
       </c>
       <c r="C588" t="str">
-        <v>J10N4yGDiUywCTAZI2lyOGUAHFjv</v>
+        <v>RDgWMx4cKUe-VTRRwOeAsWUADV42</v>
       </c>
       <c r="D588" t="str">
         <v/>
@@ -69137,6 +69196,9 @@
       </c>
       <c r="R588" t="str">
         <v>Coordination;Construction Phase</v>
+      </c>
+      <c r="S588" t="str">
+        <v>Sent out to project team, with all new elevations labeled</v>
       </c>
     </row>
     <row r="589">
@@ -69427,7 +69489,7 @@
         <v>Woonsocket Area C Level 1 Signoff</v>
       </c>
       <c r="C594" t="str">
-        <v>LfZKE0T-a0mQ-gb0hCcuzGUAM0hw</v>
+        <v>J10N4yGDiUywCTAZI2lyOGUAHFjv</v>
       </c>
       <c r="D594" t="str">
         <v/>
@@ -69448,7 +69510,7 @@
         <v>2026-06-02</v>
       </c>
       <c r="J594" t="str">
-        <v>2026-06-04</v>
+        <v>2026-06-09</v>
       </c>
       <c r="K594" t="str">
         <v/>
@@ -69495,7 +69557,7 @@
         <v>Medium</v>
       </c>
       <c r="G595" t="str">
-        <v/>
+        <v>ea3a7b10-e540-4727-a6c2-523e99fee36e</v>
       </c>
       <c r="H595" t="str">
         <v>ea3a7b10-e540-4727-a6c2-523e99fee36e</v>
@@ -69528,12 +69590,68 @@
         <v/>
       </c>
       <c r="R595" t="str">
-        <v/>
+        <v>Site Logistics;Construction Phase</v>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="str">
+        <v>uxx9CDvxYEixOsqoelK5SmUAK_4f</v>
+      </c>
+      <c r="B596" t="str">
+        <v>Glen Dr Septic As-Built</v>
+      </c>
+      <c r="C596" t="str">
+        <v>J10N4yGDiUywCTAZI2lyOGUAHFjv</v>
+      </c>
+      <c r="D596" t="str">
+        <v/>
+      </c>
+      <c r="E596" t="str">
+        <v>Not started</v>
+      </c>
+      <c r="F596" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="G596" t="str">
+        <v>4572dfb3-e99e-4bad-9d67-d344178b2d4b</v>
+      </c>
+      <c r="H596" t="str">
+        <v>f23519cd-6d4d-4cf3-8c1d-dcef0734dd79</v>
+      </c>
+      <c r="I596" t="str">
+        <v>2026-06-08</v>
+      </c>
+      <c r="J596" t="str">
+        <v/>
+      </c>
+      <c r="K596" t="str">
+        <v/>
+      </c>
+      <c r="L596" t="str">
+        <v/>
+      </c>
+      <c r="M596" t="str">
+        <v>false</v>
+      </c>
+      <c r="N596" t="str">
+        <v/>
+      </c>
+      <c r="O596" t="str">
+        <v/>
+      </c>
+      <c r="P596" t="str">
+        <v/>
+      </c>
+      <c r="Q596" t="str">
+        <v/>
+      </c>
+      <c r="R596" t="str">
+        <v>As-Built;Construction Phase</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S595"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S596"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Weekly update Tue 06/16/2026
</commit_message>
<xml_diff>
--- a/VDC Short Term Kanban.xlsx
+++ b/VDC Short Term Kanban.xlsx
@@ -428,7 +428,7 @@
         <v>VDC Short Term Kanban</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-06-08</v>
+        <v>2026-06-16</v>
       </c>
     </row>
   </sheetData>
@@ -440,7 +440,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S596"/>
+  <dimension ref="A1:S598"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -28778,7 +28778,7 @@
         <v>Modeling;Construction Phase;Process Mechanical Modeling</v>
       </c>
       <c r="S485" t="str">
-        <v>Walls adjusted, finishing up roof modeling.</v>
+        <v>More questions based on structural changes - included in Amber's email to Matt 6/11. Mostly complete, just need dimensional questions answered to finalize.</v>
       </c>
     </row>
     <row r="486">
@@ -28837,7 +28837,7 @@
         <v>Modeling;Construction Phase;Process Mechanical Modeling</v>
       </c>
       <c r="S486" t="str">
-        <v>RFIs have been submitted and returned, working through them. Approximately 50% complete.</v>
+        <v>Additional questions have been raised while modeling, email sent by Amber to Matt 6/11. Everything modeled except for roof, need questions answered to finish up.</v>
       </c>
     </row>
     <row r="487">
@@ -30873,13 +30873,13 @@
         <v>Create Model Checker Template with Autodesk Interoperability Tools</v>
       </c>
       <c r="C523" t="str">
-        <v>To do</v>
+        <v>Archive</v>
       </c>
       <c r="D523" t="str">
         <v/>
       </c>
       <c r="E523" t="str">
-        <v>Not started</v>
+        <v>Completed</v>
       </c>
       <c r="F523" t="str">
         <v>Medium</v>
@@ -30906,10 +30906,10 @@
         <v>false</v>
       </c>
       <c r="N523" t="str">
-        <v/>
+        <v>2026-06-15</v>
       </c>
       <c r="O523" t="str">
-        <v/>
+        <v>Nicholas Ambrosino</v>
       </c>
       <c r="P523" t="str">
         <v/>
@@ -32737,7 +32737,7 @@
         <v>Shaker Level 1 Signoff</v>
       </c>
       <c r="C556" t="str">
-        <v>To do</v>
+        <v>Doing</v>
       </c>
       <c r="D556" t="str">
         <v>Shaker Museum Coordination</v>
@@ -33297,13 +33297,13 @@
         <v>Congregation B'Nai Israel Logistics</v>
       </c>
       <c r="C566" t="str">
-        <v>Doing</v>
+        <v>Done</v>
       </c>
       <c r="D566" t="str">
         <v/>
       </c>
       <c r="E566" t="str">
-        <v>Not started</v>
+        <v>Completed</v>
       </c>
       <c r="F566" t="str">
         <v>Medium</v>
@@ -33330,16 +33330,16 @@
         <v>false</v>
       </c>
       <c r="N566" t="str">
-        <v/>
+        <v>2026-06-15</v>
       </c>
       <c r="O566" t="str">
-        <v/>
+        <v>Nicholas Ambrosino</v>
       </c>
       <c r="P566" t="str">
-        <v>4/4</v>
+        <v>5/5</v>
       </c>
       <c r="Q566" t="str">
-        <v>V1 - 5.5.26;V3 - 5.11.26;V0 - 5.1.26;V2 - 5.5.26</v>
+        <v>V1 - 5.5.26;V3 - 5.11.26;V0 - 5.1.26;V2 - 5.5.26;V4.1 - 6.9.26</v>
       </c>
       <c r="R566" t="str">
         <v>Site Logistics</v>
@@ -33353,13 +33353,13 @@
         <v>Marist Science Building 3D Logistics</v>
       </c>
       <c r="C567" t="str">
-        <v>Doing</v>
+        <v>Done</v>
       </c>
       <c r="D567" t="str">
         <v/>
       </c>
       <c r="E567" t="str">
-        <v>Not started</v>
+        <v>Completed</v>
       </c>
       <c r="F567" t="str">
         <v>Important</v>
@@ -33386,10 +33386,10 @@
         <v>false</v>
       </c>
       <c r="N567" t="str">
-        <v/>
+        <v>2026-06-15</v>
       </c>
       <c r="O567" t="str">
-        <v/>
+        <v>Nicholas Ambrosino</v>
       </c>
       <c r="P567" t="str">
         <v>1/2</v>
@@ -33866,7 +33866,7 @@
         <v/>
       </c>
       <c r="E576" t="str">
-        <v>Not started</v>
+        <v>Completed</v>
       </c>
       <c r="F576" t="str">
         <v>Medium</v>
@@ -33890,13 +33890,13 @@
         <v/>
       </c>
       <c r="M576" t="str">
-        <v>true</v>
+        <v>false</v>
       </c>
       <c r="N576" t="str">
-        <v/>
+        <v>2026-06-15</v>
       </c>
       <c r="O576" t="str">
-        <v/>
+        <v>Nicholas Ambrosino</v>
       </c>
       <c r="P576" t="str">
         <v/>
@@ -34034,7 +34034,7 @@
         <v/>
       </c>
       <c r="E579" t="str">
-        <v>Not started</v>
+        <v>Completed</v>
       </c>
       <c r="F579" t="str">
         <v>Urgent</v>
@@ -34061,10 +34061,10 @@
         <v>false</v>
       </c>
       <c r="N579" t="str">
-        <v/>
+        <v>2026-06-15</v>
       </c>
       <c r="O579" t="str">
-        <v/>
+        <v>Nicholas Ambrosino</v>
       </c>
       <c r="P579" t="str">
         <v>2/2</v>
@@ -34140,16 +34140,16 @@
         <v>Update Clark Logistics with new layout</v>
       </c>
       <c r="C581" t="str">
-        <v>Doing</v>
+        <v>Done</v>
       </c>
       <c r="D581" t="str">
         <v/>
       </c>
       <c r="E581" t="str">
-        <v>Not started</v>
+        <v>Completed</v>
       </c>
       <c r="F581" t="str">
-        <v>Important</v>
+        <v>Low</v>
       </c>
       <c r="G581" t="str">
         <v>Amber Webb</v>
@@ -34161,7 +34161,7 @@
         <v>2026-05-22</v>
       </c>
       <c r="J581" t="str">
-        <v>2026-06-08</v>
+        <v/>
       </c>
       <c r="K581" t="str">
         <v/>
@@ -34173,16 +34173,16 @@
         <v>false</v>
       </c>
       <c r="N581" t="str">
-        <v/>
+        <v>2026-06-15</v>
       </c>
       <c r="O581" t="str">
-        <v/>
+        <v>Nicholas Ambrosino</v>
       </c>
       <c r="P581" t="str">
-        <v/>
+        <v>2/2</v>
       </c>
       <c r="Q581" t="str">
-        <v/>
+        <v>interior V8 - 6.9.26;Exterior V9 - 6.8.26</v>
       </c>
       <c r="R581" t="str">
         <v>Site Logistics;Preconstruction</v>
@@ -34276,7 +34276,7 @@
         <v>2026-05-22</v>
       </c>
       <c r="J583" t="str">
-        <v>2026-06-12</v>
+        <v>2026-06-19</v>
       </c>
       <c r="K583" t="str">
         <v/>
@@ -34303,7 +34303,7 @@
         <v>Process Mechanical Modeling</v>
       </c>
       <c r="S583" t="str">
-        <v>Only 2 submittals for process piping are in, with 30 more to come. Mike is waiting for contract with Core and Main before we can get the rest</v>
+        <v>6.15 - Need to check with project team about where submittals are being used/what systems</v>
       </c>
     </row>
     <row r="584">
@@ -34335,7 +34335,7 @@
         <v>2026-05-22</v>
       </c>
       <c r="J584" t="str">
-        <v>2026-06-12</v>
+        <v>2026-06-19</v>
       </c>
       <c r="K584" t="str">
         <v/>
@@ -34485,7 +34485,7 @@
         <v>Low Rd Model Footing Drain</v>
       </c>
       <c r="C587" t="str">
-        <v>To do</v>
+        <v>Doing</v>
       </c>
       <c r="D587" t="str">
         <v/>
@@ -34547,7 +34547,7 @@
         <v/>
       </c>
       <c r="E588" t="str">
-        <v>Not started</v>
+        <v>Completed</v>
       </c>
       <c r="F588" t="str">
         <v>Medium</v>
@@ -34574,10 +34574,10 @@
         <v>false</v>
       </c>
       <c r="N588" t="str">
-        <v/>
+        <v>2026-06-15</v>
       </c>
       <c r="O588" t="str">
-        <v/>
+        <v>Nicholas Ambrosino</v>
       </c>
       <c r="P588" t="str">
         <v/>
@@ -34600,19 +34600,19 @@
         <v>Hazard Communication Training - 360 Learning</v>
       </c>
       <c r="C589" t="str">
-        <v>To do</v>
+        <v>Done</v>
       </c>
       <c r="D589" t="str">
         <v/>
       </c>
       <c r="E589" t="str">
-        <v>Not started</v>
+        <v>Completed</v>
       </c>
       <c r="F589" t="str">
         <v>Medium</v>
       </c>
       <c r="G589" t="str">
-        <v>Luke O'Brien;Amber Webb;Nicholas Ambrosino;Robert White</v>
+        <v>Robert White</v>
       </c>
       <c r="H589" t="str">
         <v>Amber Webb</v>
@@ -34633,10 +34633,10 @@
         <v>false</v>
       </c>
       <c r="N589" t="str">
-        <v/>
+        <v>2026-06-15</v>
       </c>
       <c r="O589" t="str">
-        <v/>
+        <v>Nicholas Ambrosino</v>
       </c>
       <c r="P589" t="str">
         <v/>
@@ -34901,7 +34901,7 @@
         <v>2026-06-02</v>
       </c>
       <c r="J594" t="str">
-        <v>2026-06-09</v>
+        <v>2026-06-16</v>
       </c>
       <c r="K594" t="str">
         <v/>
@@ -34926,6 +34926,9 @@
       </c>
       <c r="R594" t="str">
         <v>Coordination;Construction Phase</v>
+      </c>
+      <c r="S594" t="str">
+        <v>6.15 - working on this with modelers, hoping to get out for signoff today/tomorrow</v>
       </c>
     </row>
     <row r="595">
@@ -35039,17 +35042,132 @@
       <c r="R596" t="str">
         <v>As-Built;Construction Phase</v>
       </c>
+      <c r="S596" t="str">
+        <v>6.15.26 - Team reviewing updates, will let us know if any further changes reqd</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="str">
+        <v>7W9a7BW1y0GvFUQGf6oeFGUAGVy0</v>
+      </c>
+      <c r="B597" t="str">
+        <v>Willow Street Parking Logistics</v>
+      </c>
+      <c r="C597" t="str">
+        <v>Doing</v>
+      </c>
+      <c r="D597" t="str">
+        <v/>
+      </c>
+      <c r="E597" t="str">
+        <v>In progress</v>
+      </c>
+      <c r="F597" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="G597" t="str">
+        <v>Amber Webb</v>
+      </c>
+      <c r="H597" t="str">
+        <v>Amber Webb</v>
+      </c>
+      <c r="I597" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="J597" t="str">
+        <v>2026-06-16</v>
+      </c>
+      <c r="K597" t="str">
+        <v/>
+      </c>
+      <c r="L597" t="str">
+        <v/>
+      </c>
+      <c r="M597" t="str">
+        <v>false</v>
+      </c>
+      <c r="N597" t="str">
+        <v/>
+      </c>
+      <c r="O597" t="str">
+        <v/>
+      </c>
+      <c r="P597" t="str">
+        <v/>
+      </c>
+      <c r="Q597" t="str">
+        <v/>
+      </c>
+      <c r="R597" t="str">
+        <v>Site Logistics;Preconstruction</v>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="str">
+        <v>HFm8z5sWJkKSyOu4jqDKAmUAE5ly</v>
+      </c>
+      <c r="B598" t="str">
+        <v>St Paul's School Updated Design Models in Revizto</v>
+      </c>
+      <c r="C598" t="str">
+        <v>To do</v>
+      </c>
+      <c r="D598" t="str">
+        <v/>
+      </c>
+      <c r="E598" t="str">
+        <v>Not started</v>
+      </c>
+      <c r="F598" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="G598" t="str">
+        <v>Robert White</v>
+      </c>
+      <c r="H598" t="str">
+        <v>Nicholas Ambrosino</v>
+      </c>
+      <c r="I598" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="J598" t="str">
+        <v/>
+      </c>
+      <c r="K598" t="str">
+        <v/>
+      </c>
+      <c r="L598" t="str">
+        <v/>
+      </c>
+      <c r="M598" t="str">
+        <v>false</v>
+      </c>
+      <c r="N598" t="str">
+        <v/>
+      </c>
+      <c r="O598" t="str">
+        <v/>
+      </c>
+      <c r="P598" t="str">
+        <v/>
+      </c>
+      <c r="Q598" t="str">
+        <v/>
+      </c>
+      <c r="R598" t="str">
+        <v>Preconstruction;Modeling</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S596"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S598"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S596"/>
+  <dimension ref="A1:S598"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -63387,7 +63505,7 @@
         <v>Modeling;Construction Phase;Process Mechanical Modeling</v>
       </c>
       <c r="S485" t="str">
-        <v>Walls adjusted, finishing up roof modeling.</v>
+        <v>More questions based on structural changes - included in Amber's email to Matt 6/11. Mostly complete, just need dimensional questions answered to finalize.</v>
       </c>
     </row>
     <row r="486">
@@ -63446,7 +63564,7 @@
         <v>Modeling;Construction Phase;Process Mechanical Modeling</v>
       </c>
       <c r="S486" t="str">
-        <v>RFIs have been submitted and returned, working through them. Approximately 50% complete.</v>
+        <v>Additional questions have been raised while modeling, email sent by Amber to Matt 6/11. Everything modeled except for roof, need questions answered to finish up.</v>
       </c>
     </row>
     <row r="487">
@@ -65482,13 +65600,13 @@
         <v>Create Model Checker Template with Autodesk Interoperability Tools</v>
       </c>
       <c r="C523" t="str">
-        <v>LfZKE0T-a0mQ-gb0hCcuzGUAM0hw</v>
+        <v>GtpNVssKvkeVDuAfU9DPiWUAB4MO</v>
       </c>
       <c r="D523" t="str">
         <v/>
       </c>
       <c r="E523" t="str">
-        <v>Not started</v>
+        <v>Completed</v>
       </c>
       <c r="F523" t="str">
         <v>Medium</v>
@@ -65515,10 +65633,10 @@
         <v>false</v>
       </c>
       <c r="N523" t="str">
-        <v/>
+        <v>2026-06-15</v>
       </c>
       <c r="O523" t="str">
-        <v/>
+        <v>f23519cd-6d4d-4cf3-8c1d-dcef0734dd79</v>
       </c>
       <c r="P523" t="str">
         <v/>
@@ -67346,7 +67464,7 @@
         <v>Shaker Level 1 Signoff</v>
       </c>
       <c r="C556" t="str">
-        <v>LfZKE0T-a0mQ-gb0hCcuzGUAM0hw</v>
+        <v>J10N4yGDiUywCTAZI2lyOGUAHFjv</v>
       </c>
       <c r="D556" t="str">
         <v>cwPaYCpwtkKmvakyn56rG2UAGvZx</v>
@@ -67906,13 +68024,13 @@
         <v>Congregation B'Nai Israel Logistics</v>
       </c>
       <c r="C566" t="str">
-        <v>J10N4yGDiUywCTAZI2lyOGUAHFjv</v>
+        <v>RDgWMx4cKUe-VTRRwOeAsWUADV42</v>
       </c>
       <c r="D566" t="str">
         <v/>
       </c>
       <c r="E566" t="str">
-        <v>Not started</v>
+        <v>Completed</v>
       </c>
       <c r="F566" t="str">
         <v>Medium</v>
@@ -67939,16 +68057,16 @@
         <v>false</v>
       </c>
       <c r="N566" t="str">
-        <v/>
+        <v>2026-06-15</v>
       </c>
       <c r="O566" t="str">
-        <v/>
+        <v>f23519cd-6d4d-4cf3-8c1d-dcef0734dd79</v>
       </c>
       <c r="P566" t="str">
-        <v>4/4</v>
+        <v>5/5</v>
       </c>
       <c r="Q566" t="str">
-        <v>V1 - 5.5.26;V3 - 5.11.26;V0 - 5.1.26;V2 - 5.5.26</v>
+        <v>V1 - 5.5.26;V3 - 5.11.26;V0 - 5.1.26;V2 - 5.5.26;V4.1 - 6.9.26</v>
       </c>
       <c r="R566" t="str">
         <v>Site Logistics</v>
@@ -67962,13 +68080,13 @@
         <v>Marist Science Building 3D Logistics</v>
       </c>
       <c r="C567" t="str">
-        <v>J10N4yGDiUywCTAZI2lyOGUAHFjv</v>
+        <v>RDgWMx4cKUe-VTRRwOeAsWUADV42</v>
       </c>
       <c r="D567" t="str">
         <v/>
       </c>
       <c r="E567" t="str">
-        <v>Not started</v>
+        <v>Completed</v>
       </c>
       <c r="F567" t="str">
         <v>Important</v>
@@ -67995,10 +68113,10 @@
         <v>false</v>
       </c>
       <c r="N567" t="str">
-        <v/>
+        <v>2026-06-15</v>
       </c>
       <c r="O567" t="str">
-        <v/>
+        <v>f23519cd-6d4d-4cf3-8c1d-dcef0734dd79</v>
       </c>
       <c r="P567" t="str">
         <v>1/2</v>
@@ -68475,7 +68593,7 @@
         <v/>
       </c>
       <c r="E576" t="str">
-        <v>Not started</v>
+        <v>Completed</v>
       </c>
       <c r="F576" t="str">
         <v>Medium</v>
@@ -68499,13 +68617,13 @@
         <v/>
       </c>
       <c r="M576" t="str">
-        <v>true</v>
+        <v>false</v>
       </c>
       <c r="N576" t="str">
-        <v/>
+        <v>2026-06-15</v>
       </c>
       <c r="O576" t="str">
-        <v/>
+        <v>f23519cd-6d4d-4cf3-8c1d-dcef0734dd79</v>
       </c>
       <c r="P576" t="str">
         <v/>
@@ -68643,7 +68761,7 @@
         <v/>
       </c>
       <c r="E579" t="str">
-        <v>Not started</v>
+        <v>Completed</v>
       </c>
       <c r="F579" t="str">
         <v>Urgent</v>
@@ -68670,10 +68788,10 @@
         <v>false</v>
       </c>
       <c r="N579" t="str">
-        <v/>
+        <v>2026-06-15</v>
       </c>
       <c r="O579" t="str">
-        <v/>
+        <v>f23519cd-6d4d-4cf3-8c1d-dcef0734dd79</v>
       </c>
       <c r="P579" t="str">
         <v>2/2</v>
@@ -68749,16 +68867,16 @@
         <v>Update Clark Logistics with new layout</v>
       </c>
       <c r="C581" t="str">
-        <v>J10N4yGDiUywCTAZI2lyOGUAHFjv</v>
+        <v>RDgWMx4cKUe-VTRRwOeAsWUADV42</v>
       </c>
       <c r="D581" t="str">
         <v/>
       </c>
       <c r="E581" t="str">
-        <v>Not started</v>
+        <v>Completed</v>
       </c>
       <c r="F581" t="str">
-        <v>Important</v>
+        <v>Low</v>
       </c>
       <c r="G581" t="str">
         <v>ea3a7b10-e540-4727-a6c2-523e99fee36e</v>
@@ -68770,7 +68888,7 @@
         <v>2026-05-22</v>
       </c>
       <c r="J581" t="str">
-        <v>2026-06-08</v>
+        <v/>
       </c>
       <c r="K581" t="str">
         <v/>
@@ -68782,16 +68900,16 @@
         <v>false</v>
       </c>
       <c r="N581" t="str">
-        <v/>
+        <v>2026-06-15</v>
       </c>
       <c r="O581" t="str">
-        <v/>
+        <v>f23519cd-6d4d-4cf3-8c1d-dcef0734dd79</v>
       </c>
       <c r="P581" t="str">
-        <v/>
+        <v>2/2</v>
       </c>
       <c r="Q581" t="str">
-        <v/>
+        <v>interior V8 - 6.9.26;Exterior V9 - 6.8.26</v>
       </c>
       <c r="R581" t="str">
         <v>Site Logistics;Preconstruction</v>
@@ -68885,7 +69003,7 @@
         <v>2026-05-22</v>
       </c>
       <c r="J583" t="str">
-        <v>2026-06-12</v>
+        <v>2026-06-19</v>
       </c>
       <c r="K583" t="str">
         <v/>
@@ -68912,7 +69030,7 @@
         <v>Process Mechanical Modeling</v>
       </c>
       <c r="S583" t="str">
-        <v>Only 2 submittals for process piping are in, with 30 more to come. Mike is waiting for contract with Core and Main before we can get the rest</v>
+        <v>6.15 - Need to check with project team about where submittals are being used/what systems</v>
       </c>
     </row>
     <row r="584">
@@ -68944,7 +69062,7 @@
         <v>2026-05-22</v>
       </c>
       <c r="J584" t="str">
-        <v>2026-06-12</v>
+        <v>2026-06-19</v>
       </c>
       <c r="K584" t="str">
         <v/>
@@ -69094,7 +69212,7 @@
         <v>Low Rd Model Footing Drain</v>
       </c>
       <c r="C587" t="str">
-        <v>LfZKE0T-a0mQ-gb0hCcuzGUAM0hw</v>
+        <v>J10N4yGDiUywCTAZI2lyOGUAHFjv</v>
       </c>
       <c r="D587" t="str">
         <v/>
@@ -69156,7 +69274,7 @@
         <v/>
       </c>
       <c r="E588" t="str">
-        <v>Not started</v>
+        <v>Completed</v>
       </c>
       <c r="F588" t="str">
         <v>Medium</v>
@@ -69183,10 +69301,10 @@
         <v>false</v>
       </c>
       <c r="N588" t="str">
-        <v/>
+        <v>2026-06-15</v>
       </c>
       <c r="O588" t="str">
-        <v/>
+        <v>f23519cd-6d4d-4cf3-8c1d-dcef0734dd79</v>
       </c>
       <c r="P588" t="str">
         <v/>
@@ -69209,19 +69327,19 @@
         <v>Hazard Communication Training - 360 Learning</v>
       </c>
       <c r="C589" t="str">
-        <v>LfZKE0T-a0mQ-gb0hCcuzGUAM0hw</v>
+        <v>RDgWMx4cKUe-VTRRwOeAsWUADV42</v>
       </c>
       <c r="D589" t="str">
         <v/>
       </c>
       <c r="E589" t="str">
-        <v>Not started</v>
+        <v>Completed</v>
       </c>
       <c r="F589" t="str">
         <v>Medium</v>
       </c>
       <c r="G589" t="str">
-        <v>faaac610-af6d-4cd3-a69c-ddfae55ebcc4;ea3a7b10-e540-4727-a6c2-523e99fee36e;f23519cd-6d4d-4cf3-8c1d-dcef0734dd79;4572dfb3-e99e-4bad-9d67-d344178b2d4b</v>
+        <v>4572dfb3-e99e-4bad-9d67-d344178b2d4b</v>
       </c>
       <c r="H589" t="str">
         <v>ea3a7b10-e540-4727-a6c2-523e99fee36e</v>
@@ -69242,10 +69360,10 @@
         <v>false</v>
       </c>
       <c r="N589" t="str">
-        <v/>
+        <v>2026-06-15</v>
       </c>
       <c r="O589" t="str">
-        <v/>
+        <v>f23519cd-6d4d-4cf3-8c1d-dcef0734dd79</v>
       </c>
       <c r="P589" t="str">
         <v/>
@@ -69510,7 +69628,7 @@
         <v>2026-06-02</v>
       </c>
       <c r="J594" t="str">
-        <v>2026-06-09</v>
+        <v>2026-06-16</v>
       </c>
       <c r="K594" t="str">
         <v/>
@@ -69535,6 +69653,9 @@
       </c>
       <c r="R594" t="str">
         <v>Coordination;Construction Phase</v>
+      </c>
+      <c r="S594" t="str">
+        <v>6.15 - working on this with modelers, hoping to get out for signoff today/tomorrow</v>
       </c>
     </row>
     <row r="595">
@@ -69648,10 +69769,125 @@
       <c r="R596" t="str">
         <v>As-Built;Construction Phase</v>
       </c>
+      <c r="S596" t="str">
+        <v>6.15.26 - Team reviewing updates, will let us know if any further changes reqd</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="str">
+        <v>7W9a7BW1y0GvFUQGf6oeFGUAGVy0</v>
+      </c>
+      <c r="B597" t="str">
+        <v>Willow Street Parking Logistics</v>
+      </c>
+      <c r="C597" t="str">
+        <v>J10N4yGDiUywCTAZI2lyOGUAHFjv</v>
+      </c>
+      <c r="D597" t="str">
+        <v/>
+      </c>
+      <c r="E597" t="str">
+        <v>In progress</v>
+      </c>
+      <c r="F597" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="G597" t="str">
+        <v>ea3a7b10-e540-4727-a6c2-523e99fee36e</v>
+      </c>
+      <c r="H597" t="str">
+        <v>ea3a7b10-e540-4727-a6c2-523e99fee36e</v>
+      </c>
+      <c r="I597" t="str">
+        <v>2026-06-11</v>
+      </c>
+      <c r="J597" t="str">
+        <v>2026-06-16</v>
+      </c>
+      <c r="K597" t="str">
+        <v/>
+      </c>
+      <c r="L597" t="str">
+        <v/>
+      </c>
+      <c r="M597" t="str">
+        <v>false</v>
+      </c>
+      <c r="N597" t="str">
+        <v/>
+      </c>
+      <c r="O597" t="str">
+        <v/>
+      </c>
+      <c r="P597" t="str">
+        <v/>
+      </c>
+      <c r="Q597" t="str">
+        <v/>
+      </c>
+      <c r="R597" t="str">
+        <v>Site Logistics;Preconstruction</v>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="str">
+        <v>HFm8z5sWJkKSyOu4jqDKAmUAE5ly</v>
+      </c>
+      <c r="B598" t="str">
+        <v>St Paul's School Updated Design Models in Revizto</v>
+      </c>
+      <c r="C598" t="str">
+        <v>LfZKE0T-a0mQ-gb0hCcuzGUAM0hw</v>
+      </c>
+      <c r="D598" t="str">
+        <v/>
+      </c>
+      <c r="E598" t="str">
+        <v>Not started</v>
+      </c>
+      <c r="F598" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="G598" t="str">
+        <v>4572dfb3-e99e-4bad-9d67-d344178b2d4b</v>
+      </c>
+      <c r="H598" t="str">
+        <v>f23519cd-6d4d-4cf3-8c1d-dcef0734dd79</v>
+      </c>
+      <c r="I598" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="J598" t="str">
+        <v/>
+      </c>
+      <c r="K598" t="str">
+        <v/>
+      </c>
+      <c r="L598" t="str">
+        <v/>
+      </c>
+      <c r="M598" t="str">
+        <v>false</v>
+      </c>
+      <c r="N598" t="str">
+        <v/>
+      </c>
+      <c r="O598" t="str">
+        <v/>
+      </c>
+      <c r="P598" t="str">
+        <v/>
+      </c>
+      <c r="Q598" t="str">
+        <v/>
+      </c>
+      <c r="R598" t="str">
+        <v>Preconstruction;Modeling</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S596"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S598"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Weekly update Mon 06/22/2026
</commit_message>
<xml_diff>
--- a/VDC Short Term Kanban.xlsx
+++ b/VDC Short Term Kanban.xlsx
@@ -428,7 +428,7 @@
         <v>VDC Short Term Kanban</v>
       </c>
       <c r="C2" t="str">
-        <v>2026-06-16</v>
+        <v>2026-06-22</v>
       </c>
     </row>
   </sheetData>
@@ -440,7 +440,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S598"/>
+  <dimension ref="A1:S606"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -31934,6 +31934,9 @@
       <c r="R541" t="str">
         <v>Coordination;Construction Phase</v>
       </c>
+      <c r="S541" t="str">
+        <v>Restarting coordination 6/30</v>
+      </c>
     </row>
     <row r="542">
       <c r="A542" t="str">
@@ -32743,7 +32746,7 @@
         <v>Shaker Museum Coordination</v>
       </c>
       <c r="E556" t="str">
-        <v>Not started</v>
+        <v>In progress</v>
       </c>
       <c r="F556" t="str">
         <v>Medium</v>
@@ -32783,6 +32786,9 @@
       </c>
       <c r="R556" t="str">
         <v>Coordination;Construction Phase</v>
+      </c>
+      <c r="S556" t="str">
+        <v>Compiling drawings, signoff this week</v>
       </c>
     </row>
     <row r="557">
@@ -34261,7 +34267,7 @@
         <v>Bellingham WTP Coordination</v>
       </c>
       <c r="E583" t="str">
-        <v>Not started</v>
+        <v>In progress</v>
       </c>
       <c r="F583" t="str">
         <v>Medium</v>
@@ -34285,7 +34291,7 @@
         <v/>
       </c>
       <c r="M583" t="str">
-        <v>false</v>
+        <v>true</v>
       </c>
       <c r="N583" t="str">
         <v/>
@@ -34303,7 +34309,7 @@
         <v>Process Mechanical Modeling</v>
       </c>
       <c r="S583" t="str">
-        <v>6.15 - Need to check with project team about where submittals are being used/what systems</v>
+        <v>6/18 - Met with Mike Armour to go over submittal information, currently adding it to our model</v>
       </c>
     </row>
     <row r="584">
@@ -34344,7 +34350,7 @@
         <v/>
       </c>
       <c r="M584" t="str">
-        <v>false</v>
+        <v>true</v>
       </c>
       <c r="N584" t="str">
         <v/>
@@ -34491,7 +34497,7 @@
         <v/>
       </c>
       <c r="E587" t="str">
-        <v>Not started</v>
+        <v>In progress</v>
       </c>
       <c r="F587" t="str">
         <v>Medium</v>
@@ -34910,7 +34916,7 @@
         <v/>
       </c>
       <c r="M594" t="str">
-        <v>false</v>
+        <v>true</v>
       </c>
       <c r="N594" t="str">
         <v/>
@@ -34986,6 +34992,9 @@
       <c r="R595" t="str">
         <v>Site Logistics;Construction Phase</v>
       </c>
+      <c r="S595" t="str">
+        <v>Waiting on Markups from team to get started</v>
+      </c>
     </row>
     <row r="596">
       <c r="A596" t="str">
@@ -34995,7 +35004,7 @@
         <v>Glen Dr Septic As-Built</v>
       </c>
       <c r="C596" t="str">
-        <v>Doing</v>
+        <v>Done</v>
       </c>
       <c r="D596" t="str">
         <v/>
@@ -35051,10 +35060,10 @@
         <v>7W9a7BW1y0GvFUQGf6oeFGUAGVy0</v>
       </c>
       <c r="B597" t="str">
-        <v>Willow Street Parking Logistics</v>
+        <v>Willow Street Public Realm Logistics</v>
       </c>
       <c r="C597" t="str">
-        <v>Doing</v>
+        <v>To do</v>
       </c>
       <c r="D597" t="str">
         <v/>
@@ -35075,7 +35084,7 @@
         <v>2026-06-11</v>
       </c>
       <c r="J597" t="str">
-        <v>2026-06-16</v>
+        <v>2026-06-25</v>
       </c>
       <c r="K597" t="str">
         <v/>
@@ -35100,6 +35109,9 @@
       </c>
       <c r="R597" t="str">
         <v>Site Logistics;Preconstruction</v>
+      </c>
+      <c r="S597" t="str">
+        <v>Markups received from NB friday 6.19.26</v>
       </c>
     </row>
     <row r="598">
@@ -35110,13 +35122,13 @@
         <v>St Paul's School Updated Design Models in Revizto</v>
       </c>
       <c r="C598" t="str">
-        <v>To do</v>
+        <v>Done</v>
       </c>
       <c r="D598" t="str">
         <v/>
       </c>
       <c r="E598" t="str">
-        <v>Not started</v>
+        <v>Completed</v>
       </c>
       <c r="F598" t="str">
         <v>Medium</v>
@@ -35143,10 +35155,10 @@
         <v>false</v>
       </c>
       <c r="N598" t="str">
-        <v/>
+        <v>2026-06-22</v>
       </c>
       <c r="O598" t="str">
-        <v/>
+        <v>Nicholas Ambrosino</v>
       </c>
       <c r="P598" t="str">
         <v/>
@@ -35155,19 +35167,470 @@
         <v/>
       </c>
       <c r="R598" t="str">
-        <v>Preconstruction;Modeling</v>
+        <v>Modeling;Preconstruction</v>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="str">
+        <v>d9L4ZCI06k-tSsdMyHYP_WUAMt-P</v>
+      </c>
+      <c r="B599" t="str">
+        <v>Lynn 60% CD Model Review</v>
+      </c>
+      <c r="C599" t="str">
+        <v>To do</v>
+      </c>
+      <c r="D599" t="str">
+        <v/>
+      </c>
+      <c r="E599" t="str">
+        <v>Not started</v>
+      </c>
+      <c r="F599" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="G599" t="str">
+        <v/>
+      </c>
+      <c r="H599" t="str">
+        <v>Nicholas Ambrosino</v>
+      </c>
+      <c r="I599" t="str">
+        <v>2026-06-17</v>
+      </c>
+      <c r="J599" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="K599" t="str">
+        <v/>
+      </c>
+      <c r="L599" t="str">
+        <v/>
+      </c>
+      <c r="M599" t="str">
+        <v>false</v>
+      </c>
+      <c r="N599" t="str">
+        <v/>
+      </c>
+      <c r="O599" t="str">
+        <v/>
+      </c>
+      <c r="P599" t="str">
+        <v/>
+      </c>
+      <c r="Q599" t="str">
+        <v/>
+      </c>
+      <c r="R599" t="str">
+        <v>Preconstruction;Coordination</v>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="str">
+        <v>oRv6dqA4V0ekghVetKX08mUAAPb6</v>
+      </c>
+      <c r="B600" t="str">
+        <v>Compile list of costs for custom apps</v>
+      </c>
+      <c r="C600" t="str">
+        <v>To do</v>
+      </c>
+      <c r="D600" t="str">
+        <v/>
+      </c>
+      <c r="E600" t="str">
+        <v>Not started</v>
+      </c>
+      <c r="F600" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="G600" t="str">
+        <v>Nicholas Ambrosino</v>
+      </c>
+      <c r="H600" t="str">
+        <v>Nicholas Ambrosino</v>
+      </c>
+      <c r="I600" t="str">
+        <v>2026-06-18</v>
+      </c>
+      <c r="J600" t="str">
+        <v/>
+      </c>
+      <c r="K600" t="str">
+        <v/>
+      </c>
+      <c r="L600" t="str">
+        <v/>
+      </c>
+      <c r="M600" t="str">
+        <v>false</v>
+      </c>
+      <c r="N600" t="str">
+        <v/>
+      </c>
+      <c r="O600" t="str">
+        <v/>
+      </c>
+      <c r="P600" t="str">
+        <v/>
+      </c>
+      <c r="Q600" t="str">
+        <v/>
+      </c>
+      <c r="R600" t="str">
+        <v>Catalyst;AI</v>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="str">
+        <v>Mfg_nmlxWEWQWLQhtD8y2mUAFjK_</v>
+      </c>
+      <c r="B601" t="str">
+        <v>Data Comparing New PM process with previous</v>
+      </c>
+      <c r="C601" t="str">
+        <v>To do</v>
+      </c>
+      <c r="D601" t="str">
+        <v/>
+      </c>
+      <c r="E601" t="str">
+        <v>Not started</v>
+      </c>
+      <c r="F601" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="G601" t="str">
+        <v>Nicholas Ambrosino</v>
+      </c>
+      <c r="H601" t="str">
+        <v>Nicholas Ambrosino</v>
+      </c>
+      <c r="I601" t="str">
+        <v>2026-06-18</v>
+      </c>
+      <c r="J601" t="str">
+        <v/>
+      </c>
+      <c r="K601" t="str">
+        <v/>
+      </c>
+      <c r="L601" t="str">
+        <v/>
+      </c>
+      <c r="M601" t="str">
+        <v>false</v>
+      </c>
+      <c r="N601" t="str">
+        <v/>
+      </c>
+      <c r="O601" t="str">
+        <v/>
+      </c>
+      <c r="P601" t="str">
+        <v/>
+      </c>
+      <c r="Q601" t="str">
+        <v/>
+      </c>
+      <c r="R601" t="str">
+        <v>Modeling;Catalyst</v>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="str">
+        <v>_sEbyqS97ECyRDOvrupTtmUANti2</v>
+      </c>
+      <c r="B602" t="str">
+        <v>UMass Amherst Proposal Logistics - Chenoweth</v>
+      </c>
+      <c r="C602" t="str">
+        <v>Doing</v>
+      </c>
+      <c r="D602" t="str">
+        <v/>
+      </c>
+      <c r="E602" t="str">
+        <v>In progress</v>
+      </c>
+      <c r="F602" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="G602" t="str">
+        <v/>
+      </c>
+      <c r="H602" t="str">
+        <v>Amber Webb</v>
+      </c>
+      <c r="I602" t="str">
+        <v>2026-06-19</v>
+      </c>
+      <c r="J602" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="K602" t="str">
+        <v/>
+      </c>
+      <c r="L602" t="str">
+        <v/>
+      </c>
+      <c r="M602" t="str">
+        <v>false</v>
+      </c>
+      <c r="N602" t="str">
+        <v/>
+      </c>
+      <c r="O602" t="str">
+        <v/>
+      </c>
+      <c r="P602" t="str">
+        <v/>
+      </c>
+      <c r="Q602" t="str">
+        <v/>
+      </c>
+      <c r="R602" t="str">
+        <v>Site Logistics;Proposal</v>
+      </c>
+      <c r="S602" t="str">
+        <v>Markups from JW saved on Forma</v>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="str">
+        <v>LUvjkTo7DkKeqemznBZlemUAFBdq</v>
+      </c>
+      <c r="B603" t="str">
+        <v>Amherst Decarb Weekly</v>
+      </c>
+      <c r="C603" t="str">
+        <v>Drone</v>
+      </c>
+      <c r="D603" t="str">
+        <v/>
+      </c>
+      <c r="E603" t="str">
+        <v>Not started</v>
+      </c>
+      <c r="F603" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="G603" t="str">
+        <v>Luke O'Brien</v>
+      </c>
+      <c r="H603" t="str">
+        <v>Nicholas Ambrosino</v>
+      </c>
+      <c r="I603" t="str">
+        <v>2026-06-19</v>
+      </c>
+      <c r="J603" t="str">
+        <v/>
+      </c>
+      <c r="K603" t="str">
+        <v/>
+      </c>
+      <c r="L603" t="str">
+        <v/>
+      </c>
+      <c r="M603" t="str">
+        <v>false</v>
+      </c>
+      <c r="N603" t="str">
+        <v/>
+      </c>
+      <c r="O603" t="str">
+        <v/>
+      </c>
+      <c r="P603" t="str">
+        <v/>
+      </c>
+      <c r="Q603" t="str">
+        <v/>
+      </c>
+      <c r="R603" t="str">
+        <v>Drone</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="str">
+        <v>fuazTVIUpkKlHaQtZuW_mWUABut1</v>
+      </c>
+      <c r="B604" t="str">
+        <v>Trinity Decarb Weekly</v>
+      </c>
+      <c r="C604" t="str">
+        <v>Drone</v>
+      </c>
+      <c r="D604" t="str">
+        <v/>
+      </c>
+      <c r="E604" t="str">
+        <v>Not started</v>
+      </c>
+      <c r="F604" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="G604" t="str">
+        <v>Nicholas Ambrosino</v>
+      </c>
+      <c r="H604" t="str">
+        <v>Nicholas Ambrosino</v>
+      </c>
+      <c r="I604" t="str">
+        <v>2026-06-19</v>
+      </c>
+      <c r="J604" t="str">
+        <v/>
+      </c>
+      <c r="K604" t="str">
+        <v/>
+      </c>
+      <c r="L604" t="str">
+        <v/>
+      </c>
+      <c r="M604" t="str">
+        <v>false</v>
+      </c>
+      <c r="N604" t="str">
+        <v/>
+      </c>
+      <c r="O604" t="str">
+        <v/>
+      </c>
+      <c r="P604" t="str">
+        <v/>
+      </c>
+      <c r="Q604" t="str">
+        <v/>
+      </c>
+      <c r="R604" t="str">
+        <v>Drone</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="str">
+        <v>jkoh6hvI4U-Mae7su3cVgGUANp-t</v>
+      </c>
+      <c r="B605" t="str">
+        <v>Leicester High Logistics</v>
+      </c>
+      <c r="C605" t="str">
+        <v>Doing</v>
+      </c>
+      <c r="D605" t="str">
+        <v/>
+      </c>
+      <c r="E605" t="str">
+        <v>In progress</v>
+      </c>
+      <c r="F605" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="G605" t="str">
+        <v>Amber Webb</v>
+      </c>
+      <c r="H605" t="str">
+        <v>Amber Webb</v>
+      </c>
+      <c r="I605" t="str">
+        <v>2026-06-19</v>
+      </c>
+      <c r="J605" t="str">
+        <v>2026-06-23</v>
+      </c>
+      <c r="K605" t="str">
+        <v/>
+      </c>
+      <c r="L605" t="str">
+        <v/>
+      </c>
+      <c r="M605" t="str">
+        <v>false</v>
+      </c>
+      <c r="N605" t="str">
+        <v/>
+      </c>
+      <c r="O605" t="str">
+        <v/>
+      </c>
+      <c r="P605" t="str">
+        <v>0/1</v>
+      </c>
+      <c r="Q605" t="str">
+        <v>V1-6.19.26</v>
+      </c>
+      <c r="R605" t="str">
+        <v>Site Logistics;Proposal</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="str">
+        <v>riltThA2QUCcE3veePg2U2UAFdBB</v>
+      </c>
+      <c r="B606" t="str">
+        <v>Collier County WRF MBR Underground Piping Model</v>
+      </c>
+      <c r="C606" t="str">
+        <v>To do</v>
+      </c>
+      <c r="D606" t="str">
+        <v/>
+      </c>
+      <c r="E606" t="str">
+        <v>Not started</v>
+      </c>
+      <c r="F606" t="str">
+        <v>Important</v>
+      </c>
+      <c r="G606" t="str">
+        <v/>
+      </c>
+      <c r="H606" t="str">
+        <v>Nicholas Ambrosino</v>
+      </c>
+      <c r="I606" t="str">
+        <v>2026-06-22</v>
+      </c>
+      <c r="J606" t="str">
+        <v>2026-07-17</v>
+      </c>
+      <c r="K606" t="str">
+        <v/>
+      </c>
+      <c r="L606" t="str">
+        <v/>
+      </c>
+      <c r="M606" t="str">
+        <v>false</v>
+      </c>
+      <c r="N606" t="str">
+        <v/>
+      </c>
+      <c r="O606" t="str">
+        <v/>
+      </c>
+      <c r="P606" t="str">
+        <v/>
+      </c>
+      <c r="Q606" t="str">
+        <v/>
+      </c>
+      <c r="R606" t="str">
+        <v>Coordination;Construction Phase;Process Mechanical Modeling</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S598"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S606"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S598"/>
+  <dimension ref="A1:S606"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -66661,6 +67124,9 @@
       <c r="R541" t="str">
         <v>Coordination;Construction Phase</v>
       </c>
+      <c r="S541" t="str">
+        <v>Restarting coordination 6/30</v>
+      </c>
     </row>
     <row r="542">
       <c r="A542" t="str">
@@ -67470,7 +67936,7 @@
         <v>cwPaYCpwtkKmvakyn56rG2UAGvZx</v>
       </c>
       <c r="E556" t="str">
-        <v>Not started</v>
+        <v>In progress</v>
       </c>
       <c r="F556" t="str">
         <v>Medium</v>
@@ -67510,6 +67976,9 @@
       </c>
       <c r="R556" t="str">
         <v>Coordination;Construction Phase</v>
+      </c>
+      <c r="S556" t="str">
+        <v>Compiling drawings, signoff this week</v>
       </c>
     </row>
     <row r="557">
@@ -68988,7 +69457,7 @@
         <v>dBoM6XO39EuPBFSA8gEBJmUAEiyN</v>
       </c>
       <c r="E583" t="str">
-        <v>Not started</v>
+        <v>In progress</v>
       </c>
       <c r="F583" t="str">
         <v>Medium</v>
@@ -69012,7 +69481,7 @@
         <v/>
       </c>
       <c r="M583" t="str">
-        <v>false</v>
+        <v>true</v>
       </c>
       <c r="N583" t="str">
         <v/>
@@ -69030,7 +69499,7 @@
         <v>Process Mechanical Modeling</v>
       </c>
       <c r="S583" t="str">
-        <v>6.15 - Need to check with project team about where submittals are being used/what systems</v>
+        <v>6/18 - Met with Mike Armour to go over submittal information, currently adding it to our model</v>
       </c>
     </row>
     <row r="584">
@@ -69071,7 +69540,7 @@
         <v/>
       </c>
       <c r="M584" t="str">
-        <v>false</v>
+        <v>true</v>
       </c>
       <c r="N584" t="str">
         <v/>
@@ -69218,7 +69687,7 @@
         <v/>
       </c>
       <c r="E587" t="str">
-        <v>Not started</v>
+        <v>In progress</v>
       </c>
       <c r="F587" t="str">
         <v>Medium</v>
@@ -69637,7 +70106,7 @@
         <v/>
       </c>
       <c r="M594" t="str">
-        <v>false</v>
+        <v>true</v>
       </c>
       <c r="N594" t="str">
         <v/>
@@ -69713,6 +70182,9 @@
       <c r="R595" t="str">
         <v>Site Logistics;Construction Phase</v>
       </c>
+      <c r="S595" t="str">
+        <v>Waiting on Markups from team to get started</v>
+      </c>
     </row>
     <row r="596">
       <c r="A596" t="str">
@@ -69722,7 +70194,7 @@
         <v>Glen Dr Septic As-Built</v>
       </c>
       <c r="C596" t="str">
-        <v>J10N4yGDiUywCTAZI2lyOGUAHFjv</v>
+        <v>RDgWMx4cKUe-VTRRwOeAsWUADV42</v>
       </c>
       <c r="D596" t="str">
         <v/>
@@ -69778,10 +70250,10 @@
         <v>7W9a7BW1y0GvFUQGf6oeFGUAGVy0</v>
       </c>
       <c r="B597" t="str">
-        <v>Willow Street Parking Logistics</v>
+        <v>Willow Street Public Realm Logistics</v>
       </c>
       <c r="C597" t="str">
-        <v>J10N4yGDiUywCTAZI2lyOGUAHFjv</v>
+        <v>LfZKE0T-a0mQ-gb0hCcuzGUAM0hw</v>
       </c>
       <c r="D597" t="str">
         <v/>
@@ -69802,7 +70274,7 @@
         <v>2026-06-11</v>
       </c>
       <c r="J597" t="str">
-        <v>2026-06-16</v>
+        <v>2026-06-25</v>
       </c>
       <c r="K597" t="str">
         <v/>
@@ -69827,6 +70299,9 @@
       </c>
       <c r="R597" t="str">
         <v>Site Logistics;Preconstruction</v>
+      </c>
+      <c r="S597" t="str">
+        <v>Markups received from NB friday 6.19.26</v>
       </c>
     </row>
     <row r="598">
@@ -69837,13 +70312,13 @@
         <v>St Paul's School Updated Design Models in Revizto</v>
       </c>
       <c r="C598" t="str">
-        <v>LfZKE0T-a0mQ-gb0hCcuzGUAM0hw</v>
+        <v>RDgWMx4cKUe-VTRRwOeAsWUADV42</v>
       </c>
       <c r="D598" t="str">
         <v/>
       </c>
       <c r="E598" t="str">
-        <v>Not started</v>
+        <v>Completed</v>
       </c>
       <c r="F598" t="str">
         <v>Medium</v>
@@ -69870,10 +70345,10 @@
         <v>false</v>
       </c>
       <c r="N598" t="str">
-        <v/>
+        <v>2026-06-22</v>
       </c>
       <c r="O598" t="str">
-        <v/>
+        <v>f23519cd-6d4d-4cf3-8c1d-dcef0734dd79</v>
       </c>
       <c r="P598" t="str">
         <v/>
@@ -69882,12 +70357,463 @@
         <v/>
       </c>
       <c r="R598" t="str">
-        <v>Preconstruction;Modeling</v>
+        <v>Modeling;Preconstruction</v>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="str">
+        <v>d9L4ZCI06k-tSsdMyHYP_WUAMt-P</v>
+      </c>
+      <c r="B599" t="str">
+        <v>Lynn 60% CD Model Review</v>
+      </c>
+      <c r="C599" t="str">
+        <v>LfZKE0T-a0mQ-gb0hCcuzGUAM0hw</v>
+      </c>
+      <c r="D599" t="str">
+        <v/>
+      </c>
+      <c r="E599" t="str">
+        <v>Not started</v>
+      </c>
+      <c r="F599" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="G599" t="str">
+        <v/>
+      </c>
+      <c r="H599" t="str">
+        <v>f23519cd-6d4d-4cf3-8c1d-dcef0734dd79</v>
+      </c>
+      <c r="I599" t="str">
+        <v>2026-06-17</v>
+      </c>
+      <c r="J599" t="str">
+        <v>2026-07-01</v>
+      </c>
+      <c r="K599" t="str">
+        <v/>
+      </c>
+      <c r="L599" t="str">
+        <v/>
+      </c>
+      <c r="M599" t="str">
+        <v>false</v>
+      </c>
+      <c r="N599" t="str">
+        <v/>
+      </c>
+      <c r="O599" t="str">
+        <v/>
+      </c>
+      <c r="P599" t="str">
+        <v/>
+      </c>
+      <c r="Q599" t="str">
+        <v/>
+      </c>
+      <c r="R599" t="str">
+        <v>Preconstruction;Coordination</v>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="str">
+        <v>oRv6dqA4V0ekghVetKX08mUAAPb6</v>
+      </c>
+      <c r="B600" t="str">
+        <v>Compile list of costs for custom apps</v>
+      </c>
+      <c r="C600" t="str">
+        <v>LfZKE0T-a0mQ-gb0hCcuzGUAM0hw</v>
+      </c>
+      <c r="D600" t="str">
+        <v/>
+      </c>
+      <c r="E600" t="str">
+        <v>Not started</v>
+      </c>
+      <c r="F600" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="G600" t="str">
+        <v>f23519cd-6d4d-4cf3-8c1d-dcef0734dd79</v>
+      </c>
+      <c r="H600" t="str">
+        <v>f23519cd-6d4d-4cf3-8c1d-dcef0734dd79</v>
+      </c>
+      <c r="I600" t="str">
+        <v>2026-06-18</v>
+      </c>
+      <c r="J600" t="str">
+        <v/>
+      </c>
+      <c r="K600" t="str">
+        <v/>
+      </c>
+      <c r="L600" t="str">
+        <v/>
+      </c>
+      <c r="M600" t="str">
+        <v>false</v>
+      </c>
+      <c r="N600" t="str">
+        <v/>
+      </c>
+      <c r="O600" t="str">
+        <v/>
+      </c>
+      <c r="P600" t="str">
+        <v/>
+      </c>
+      <c r="Q600" t="str">
+        <v/>
+      </c>
+      <c r="R600" t="str">
+        <v>Catalyst;AI</v>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="str">
+        <v>Mfg_nmlxWEWQWLQhtD8y2mUAFjK_</v>
+      </c>
+      <c r="B601" t="str">
+        <v>Data Comparing New PM process with previous</v>
+      </c>
+      <c r="C601" t="str">
+        <v>LfZKE0T-a0mQ-gb0hCcuzGUAM0hw</v>
+      </c>
+      <c r="D601" t="str">
+        <v/>
+      </c>
+      <c r="E601" t="str">
+        <v>Not started</v>
+      </c>
+      <c r="F601" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="G601" t="str">
+        <v>f23519cd-6d4d-4cf3-8c1d-dcef0734dd79</v>
+      </c>
+      <c r="H601" t="str">
+        <v>f23519cd-6d4d-4cf3-8c1d-dcef0734dd79</v>
+      </c>
+      <c r="I601" t="str">
+        <v>2026-06-18</v>
+      </c>
+      <c r="J601" t="str">
+        <v/>
+      </c>
+      <c r="K601" t="str">
+        <v/>
+      </c>
+      <c r="L601" t="str">
+        <v/>
+      </c>
+      <c r="M601" t="str">
+        <v>false</v>
+      </c>
+      <c r="N601" t="str">
+        <v/>
+      </c>
+      <c r="O601" t="str">
+        <v/>
+      </c>
+      <c r="P601" t="str">
+        <v/>
+      </c>
+      <c r="Q601" t="str">
+        <v/>
+      </c>
+      <c r="R601" t="str">
+        <v>Modeling;Catalyst</v>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="str">
+        <v>_sEbyqS97ECyRDOvrupTtmUANti2</v>
+      </c>
+      <c r="B602" t="str">
+        <v>UMass Amherst Proposal Logistics - Chenoweth</v>
+      </c>
+      <c r="C602" t="str">
+        <v>J10N4yGDiUywCTAZI2lyOGUAHFjv</v>
+      </c>
+      <c r="D602" t="str">
+        <v/>
+      </c>
+      <c r="E602" t="str">
+        <v>In progress</v>
+      </c>
+      <c r="F602" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="G602" t="str">
+        <v/>
+      </c>
+      <c r="H602" t="str">
+        <v>ea3a7b10-e540-4727-a6c2-523e99fee36e</v>
+      </c>
+      <c r="I602" t="str">
+        <v>2026-06-19</v>
+      </c>
+      <c r="J602" t="str">
+        <v>2026-06-26</v>
+      </c>
+      <c r="K602" t="str">
+        <v/>
+      </c>
+      <c r="L602" t="str">
+        <v/>
+      </c>
+      <c r="M602" t="str">
+        <v>false</v>
+      </c>
+      <c r="N602" t="str">
+        <v/>
+      </c>
+      <c r="O602" t="str">
+        <v/>
+      </c>
+      <c r="P602" t="str">
+        <v/>
+      </c>
+      <c r="Q602" t="str">
+        <v/>
+      </c>
+      <c r="R602" t="str">
+        <v>Site Logistics;Proposal</v>
+      </c>
+      <c r="S602" t="str">
+        <v>Markups from JW saved on Forma</v>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="str">
+        <v>LUvjkTo7DkKeqemznBZlemUAFBdq</v>
+      </c>
+      <c r="B603" t="str">
+        <v>Amherst Decarb Weekly</v>
+      </c>
+      <c r="C603" t="str">
+        <v>j1rkmaQZ4EKzaoo6WltlhWUAD3GJ</v>
+      </c>
+      <c r="D603" t="str">
+        <v/>
+      </c>
+      <c r="E603" t="str">
+        <v>Not started</v>
+      </c>
+      <c r="F603" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="G603" t="str">
+        <v>faaac610-af6d-4cd3-a69c-ddfae55ebcc4</v>
+      </c>
+      <c r="H603" t="str">
+        <v>f23519cd-6d4d-4cf3-8c1d-dcef0734dd79</v>
+      </c>
+      <c r="I603" t="str">
+        <v>2026-06-19</v>
+      </c>
+      <c r="J603" t="str">
+        <v/>
+      </c>
+      <c r="K603" t="str">
+        <v/>
+      </c>
+      <c r="L603" t="str">
+        <v/>
+      </c>
+      <c r="M603" t="str">
+        <v>false</v>
+      </c>
+      <c r="N603" t="str">
+        <v/>
+      </c>
+      <c r="O603" t="str">
+        <v/>
+      </c>
+      <c r="P603" t="str">
+        <v/>
+      </c>
+      <c r="Q603" t="str">
+        <v/>
+      </c>
+      <c r="R603" t="str">
+        <v>Drone</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="str">
+        <v>fuazTVIUpkKlHaQtZuW_mWUABut1</v>
+      </c>
+      <c r="B604" t="str">
+        <v>Trinity Decarb Weekly</v>
+      </c>
+      <c r="C604" t="str">
+        <v>j1rkmaQZ4EKzaoo6WltlhWUAD3GJ</v>
+      </c>
+      <c r="D604" t="str">
+        <v/>
+      </c>
+      <c r="E604" t="str">
+        <v>Not started</v>
+      </c>
+      <c r="F604" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="G604" t="str">
+        <v>f23519cd-6d4d-4cf3-8c1d-dcef0734dd79</v>
+      </c>
+      <c r="H604" t="str">
+        <v>f23519cd-6d4d-4cf3-8c1d-dcef0734dd79</v>
+      </c>
+      <c r="I604" t="str">
+        <v>2026-06-19</v>
+      </c>
+      <c r="J604" t="str">
+        <v/>
+      </c>
+      <c r="K604" t="str">
+        <v/>
+      </c>
+      <c r="L604" t="str">
+        <v/>
+      </c>
+      <c r="M604" t="str">
+        <v>false</v>
+      </c>
+      <c r="N604" t="str">
+        <v/>
+      </c>
+      <c r="O604" t="str">
+        <v/>
+      </c>
+      <c r="P604" t="str">
+        <v/>
+      </c>
+      <c r="Q604" t="str">
+        <v/>
+      </c>
+      <c r="R604" t="str">
+        <v>Drone</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="str">
+        <v>jkoh6hvI4U-Mae7su3cVgGUANp-t</v>
+      </c>
+      <c r="B605" t="str">
+        <v>Leicester High Logistics</v>
+      </c>
+      <c r="C605" t="str">
+        <v>J10N4yGDiUywCTAZI2lyOGUAHFjv</v>
+      </c>
+      <c r="D605" t="str">
+        <v/>
+      </c>
+      <c r="E605" t="str">
+        <v>In progress</v>
+      </c>
+      <c r="F605" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="G605" t="str">
+        <v>ea3a7b10-e540-4727-a6c2-523e99fee36e</v>
+      </c>
+      <c r="H605" t="str">
+        <v>ea3a7b10-e540-4727-a6c2-523e99fee36e</v>
+      </c>
+      <c r="I605" t="str">
+        <v>2026-06-19</v>
+      </c>
+      <c r="J605" t="str">
+        <v>2026-06-23</v>
+      </c>
+      <c r="K605" t="str">
+        <v/>
+      </c>
+      <c r="L605" t="str">
+        <v/>
+      </c>
+      <c r="M605" t="str">
+        <v>false</v>
+      </c>
+      <c r="N605" t="str">
+        <v/>
+      </c>
+      <c r="O605" t="str">
+        <v/>
+      </c>
+      <c r="P605" t="str">
+        <v>0/1</v>
+      </c>
+      <c r="Q605" t="str">
+        <v>V1-6.19.26</v>
+      </c>
+      <c r="R605" t="str">
+        <v>Site Logistics;Proposal</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="str">
+        <v>riltThA2QUCcE3veePg2U2UAFdBB</v>
+      </c>
+      <c r="B606" t="str">
+        <v>Collier County WRF MBR Underground Piping Model</v>
+      </c>
+      <c r="C606" t="str">
+        <v>LfZKE0T-a0mQ-gb0hCcuzGUAM0hw</v>
+      </c>
+      <c r="D606" t="str">
+        <v/>
+      </c>
+      <c r="E606" t="str">
+        <v>Not started</v>
+      </c>
+      <c r="F606" t="str">
+        <v>Important</v>
+      </c>
+      <c r="G606" t="str">
+        <v/>
+      </c>
+      <c r="H606" t="str">
+        <v>f23519cd-6d4d-4cf3-8c1d-dcef0734dd79</v>
+      </c>
+      <c r="I606" t="str">
+        <v>2026-06-22</v>
+      </c>
+      <c r="J606" t="str">
+        <v>2026-07-17</v>
+      </c>
+      <c r="K606" t="str">
+        <v/>
+      </c>
+      <c r="L606" t="str">
+        <v/>
+      </c>
+      <c r="M606" t="str">
+        <v>false</v>
+      </c>
+      <c r="N606" t="str">
+        <v/>
+      </c>
+      <c r="O606" t="str">
+        <v/>
+      </c>
+      <c r="P606" t="str">
+        <v/>
+      </c>
+      <c r="Q606" t="str">
+        <v/>
+      </c>
+      <c r="R606" t="str">
+        <v>Coordination;Construction Phase;Process Mechanical Modeling</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S598"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S606"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -70201,7 +71127,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B8"/>
   <cols>
     <col min="1" max="1" width="32.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -70263,9 +71189,17 @@
         <v>AI Projects</v>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>j1rkmaQZ4EKzaoo6WltlhWUAD3GJ</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Drone</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>